<commit_message>
feat: set up interviews
</commit_message>
<xml_diff>
--- a/test-suite/results_manual.xlsx
+++ b/test-suite/results_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ellio\Documents\MCT\AJ2025-2026\bachelorproef\thesis_research\test-suite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DEFD3E-C6D6-42EA-AD2F-CE9219CF91DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2B06C14-328B-446F-8332-79D833709E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0474721D-4CA8-47AC-98F8-0E8C5C68D0C3}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="115">
   <si>
     <t>Code</t>
   </si>
@@ -1806,7 +1806,9 @@
       <c r="H31" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="I31" s="13"/>
+      <c r="I31" s="13" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
@@ -1921,7 +1923,7 @@
       </c>
       <c r="I36" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>87.097%</v>
+        <v>87.5%</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>